<commit_message>
- examples applying the model to real zooplankton data at Station ALOHA added - template code for real zooplankton data - data files updated to include ID column - post_extract function update to exclude depricated TDF posterior object
</commit_message>
<xml_diff>
--- a/Data/OMSM_Data_Template.xlsx
+++ b/Data/OMSM_Data_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/40c9661624813381/Documents/R/Organic-Matter-Supply-Model/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="8_{980B29BF-4572-4C82-B031-9BE11627A6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3061BBB-5EF9-4213-A4F8-6527CD7281FB}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="8_{980B29BF-4572-4C82-B031-9BE11627A6F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD0B25B4-8FD0-4578-8D60-0786EF684634}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{7732368E-59F4-4971-9DE6-B46B126306AF}"/>
   </bookViews>
@@ -37,14 +37,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
   <si>
     <t>Type</t>
   </si>
   <si>
-    <t>Group</t>
-  </si>
-  <si>
     <t>…</t>
   </si>
   <si>
@@ -81,9 +78,6 @@
     <t>description</t>
   </si>
   <si>
-    <t>"source" or "consumer"</t>
-  </si>
-  <si>
     <t>text</t>
   </si>
   <si>
@@ -123,13 +117,25 @@
     <t>Source groups may also be defined programatically within the "Processing_Data" chunk. If so, leave this column blank.</t>
   </si>
   <si>
-    <t>For consumers, just enter "consumer".</t>
-  </si>
-  <si>
     <t>Defines if this row containes data for an organic matter source or for a consumer sample.</t>
   </si>
   <si>
     <t>If organic matter source, enter "Source". If consumer, enter "Consumer".</t>
+  </si>
+  <si>
+    <t>For consumers, enter "consumer" or a more specific identifier for each sample.</t>
+  </si>
+  <si>
+    <t>"Source" or "Consumer"</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Contains a unique identifier for each sample.</t>
   </si>
 </sst>
 </file>
@@ -183,7 +189,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -238,6 +244,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -259,6 +276,15 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -301,15 +327,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -654,135 +673,146 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F097B39D-6D67-4EE0-8D1A-804DB7AD32B7}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="2" max="2" width="21.5" customWidth="1"/>
-    <col min="3" max="3" width="137.04296875" customWidth="1"/>
+    <col min="3" max="3" width="147.86328125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.75">
       <c r="A1" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="C1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="12" t="s">
+    </row>
+    <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A2" s="33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="33" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A3" s="30"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="17" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A4" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="29" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A2" s="31" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="31" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="32" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" s="30" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A3" s="27"/>
-      <c r="B3" s="27"/>
-      <c r="C3" s="33" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A4" s="26" t="s">
-        <v>1</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>15</v>
-      </c>
       <c r="C4" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="5" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A5" s="26"/>
-      <c r="B5" s="26"/>
+      <c r="A5" s="29"/>
+      <c r="B5" s="29"/>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27"/>
+      <c r="A6" s="30"/>
+      <c r="B6" s="30"/>
       <c r="C6" s="13" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A7" s="28" t="s">
+    <row r="7" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A7" s="18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A8" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A9" s="32"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="20"/>
+    </row>
+    <row r="10" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A10" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="16" t="s">
+      <c r="B10" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="27" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A11" s="26"/>
+      <c r="B11" s="26"/>
+      <c r="C11" s="28"/>
+    </row>
+    <row r="12" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A12" s="21" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A8" s="29"/>
-      <c r="B8" s="29"/>
-      <c r="C8" s="17"/>
-    </row>
-    <row r="9" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A9" s="22" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" s="14" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="25"/>
-    </row>
-    <row r="11" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A11" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="20" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.75">
-      <c r="A12" s="19"/>
-      <c r="B12" s="19"/>
-      <c r="C12" s="21"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.75">
-      <c r="C13" t="s">
-        <v>25</v>
+      <c r="B12" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.75">
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="24"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="C14" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="B4:B6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="B12:B13"/>
+    <mergeCell ref="C12:C13"/>
+    <mergeCell ref="A10:A11"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -790,55 +820,57 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C326DE9-3ADE-4768-BFF1-E37E19802DD1}">
-  <dimension ref="A1:AN1"/>
+  <dimension ref="A1:AO1"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <cols>
-    <col min="1" max="1" width="6.453125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="6.453125" style="2" customWidth="1"/>
-    <col min="3" max="11" width="8.26953125" style="3" customWidth="1"/>
-    <col min="12" max="12" width="8.26953125" style="4" customWidth="1"/>
-    <col min="13" max="26" width="6.953125" style="14" customWidth="1"/>
-    <col min="27" max="40" width="9.36328125" style="5" customWidth="1"/>
+    <col min="1" max="2" width="6.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="6.453125" style="2" customWidth="1"/>
+    <col min="4" max="12" width="8.26953125" style="3" customWidth="1"/>
+    <col min="13" max="13" width="8.26953125" style="4" customWidth="1"/>
+    <col min="14" max="27" width="6.953125" style="14" customWidth="1"/>
+    <col min="28" max="41" width="9.36328125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:40" s="11" customFormat="1" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
+    <row r="1" spans="1:41" s="11" customFormat="1" ht="15.5" thickBot="1" x14ac:dyDescent="0.9">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G1" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="F1" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="G1" s="8"/>
       <c r="H1" s="8"/>
       <c r="I1" s="8"/>
       <c r="J1" s="8"/>
       <c r="K1" s="8"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="15" t="s">
+      <c r="L1" s="8"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="O1" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="P1" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="O1" s="15" t="s">
-        <v>8</v>
-      </c>
-      <c r="P1" s="15" t="s">
-        <v>2</v>
-      </c>
-      <c r="Q1" s="15"/>
+      <c r="Q1" s="15" t="s">
+        <v>1</v>
+      </c>
       <c r="R1" s="15"/>
       <c r="S1" s="15"/>
       <c r="T1" s="15"/>
@@ -848,19 +880,19 @@
       <c r="X1" s="15"/>
       <c r="Y1" s="15"/>
       <c r="Z1" s="15"/>
-      <c r="AA1" s="10" t="s">
+      <c r="AA1" s="15"/>
+      <c r="AB1" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="AC1" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="AD1" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="AB1" s="10" t="s">
-        <v>22</v>
-      </c>
-      <c r="AC1" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="AD1" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="AE1" s="10"/>
+      <c r="AE1" s="10" t="s">
+        <v>1</v>
+      </c>
       <c r="AF1" s="10"/>
       <c r="AG1" s="10"/>
       <c r="AH1" s="10"/>
@@ -870,6 +902,7 @@
       <c r="AL1" s="10"/>
       <c r="AM1" s="10"/>
       <c r="AN1" s="10"/>
+      <c r="AO1" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>